<commit_message>
ADD: FOTOS DE EXCEL BETA
</commit_message>
<xml_diff>
--- a/ProyectoVisitas/wwwroot/Templates/ListaDeAsistencia.xlsx
+++ b/ProyectoVisitas/wwwroot/Templates/ListaDeAsistencia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\ProyectoVisitas\ProyectoVisitas\wwwroot\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16220A4E-4FCC-4365-92D0-7A4EF3199318}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DA4695A-07D4-4C60-91C5-342FEC49D49D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>NO.</t>
   </si>
@@ -59,9 +59,6 @@
   </si>
   <si>
     <t>DOMICILIO Y RESPONSABLE:                                                                                                     Responsable: LIC. Blanca Pacheco                                                         Domicilio: Blvd. Miguel de Cervantes Saavedra #8701 Col. Colinas de Santa Julia</t>
-  </si>
-  <si>
-    <t>FECHA                               FOLIO</t>
   </si>
   <si>
     <t xml:space="preserve">      LISTA ASISTENCIA DE JUZGADO CÍVICO </t>
@@ -361,9 +358,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -378,6 +372,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -864,7 +861,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="22" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B1" s="22"/>
       <c r="C1" s="22"/>
@@ -879,12 +876,10 @@
       </c>
       <c r="B2" s="23"/>
       <c r="C2" s="23"/>
-      <c r="D2" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
     </row>
     <row r="3" spans="1:7" s="5" customFormat="1" ht="24" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
@@ -1064,14 +1059,14 @@
       <c r="G17" s="3"/>
     </row>
     <row r="18" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="26"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
       <c r="G18" s="11"/>
     </row>
     <row r="19" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1084,15 +1079,15 @@
       <c r="G19" s="12"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="29"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="28"/>
     </row>
     <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="18"/>

</xml_diff>

<commit_message>
ADD: Fotografias final de excel
</commit_message>
<xml_diff>
--- a/ProyectoVisitas/wwwroot/Templates/ListaDeAsistencia.xlsx
+++ b/ProyectoVisitas/wwwroot/Templates/ListaDeAsistencia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\ProyectoVisitas\ProyectoVisitas\wwwroot\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DA4695A-07D4-4C60-91C5-342FEC49D49D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C199ADF-8C70-4F41-A966-BE01ECC9D0B2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,6 +358,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -372,9 +375,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -851,10 +851,10 @@
   <cols>
     <col min="1" max="1" width="4.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="45.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="7.5703125" style="5" customWidth="1"/>
-    <col min="4" max="4" width="9" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.140625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="6.28515625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" style="5" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" style="5" customWidth="1"/>
     <col min="7" max="7" width="27.7109375" style="1" customWidth="1"/>
     <col min="8" max="16384" width="11.42578125" style="1"/>
   </cols>
@@ -876,10 +876,10 @@
       </c>
       <c r="B2" s="23"/>
       <c r="C2" s="23"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
     </row>
     <row r="3" spans="1:7" s="5" customFormat="1" ht="24" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
@@ -1059,14 +1059,14 @@
       <c r="G17" s="3"/>
     </row>
     <row r="18" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="24" t="s">
+      <c r="A18" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
       <c r="G18" s="11"/>
     </row>
     <row r="19" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1079,15 +1079,15 @@
       <c r="G19" s="12"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="26" t="s">
+      <c r="A20" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="28"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="29"/>
     </row>
     <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="18"/>

</xml_diff>